<commit_message>
Added and cleaned up some results in powerpoint
</commit_message>
<xml_diff>
--- a/results/concurrency/ConcurrencyActualResults.xlsx
+++ b/results/concurrency/ConcurrencyActualResults.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\audricho\Documents\ForOfficialDemo\results\concurrency\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6CFA079-E045-4A44-947B-1CDDC31C8B73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78B1E355-37DF-4DC7-959C-AEAC66D832D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -605,7 +605,7 @@
     <col min="5" max="19" width="13.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="75.599999999999994" customHeight="1">
+    <row r="1" spans="1:19" ht="87.6" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4401,7 +4401,7 @@
         <v>3.4418519014461704</v>
       </c>
     </row>
-    <row r="81" spans="1:4">
+    <row r="81" spans="1:11">
       <c r="A81" s="1" t="s">
         <v>5</v>
       </c>
@@ -4409,7 +4409,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="82" spans="1:4">
+    <row r="82" spans="1:11">
       <c r="A82" s="1" t="s">
         <v>6</v>
       </c>
@@ -4417,7 +4417,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="83" spans="1:4">
+    <row r="83" spans="1:11">
       <c r="A83" s="1" t="s">
         <v>7</v>
       </c>
@@ -4425,7 +4425,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="84" spans="1:4">
+    <row r="84" spans="1:11">
       <c r="A84" s="1" t="s">
         <v>8</v>
       </c>
@@ -4436,7 +4436,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="85" spans="1:4">
+    <row r="85" spans="1:11">
       <c r="A85" s="1" t="s">
         <v>9</v>
       </c>
@@ -4447,7 +4447,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="86" spans="1:4">
+    <row r="86" spans="1:11">
       <c r="A86" s="1" t="s">
         <v>10</v>
       </c>
@@ -4458,7 +4458,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="87" spans="1:4">
+    <row r="87" spans="1:11">
       <c r="A87" s="1" t="s">
         <v>11</v>
       </c>
@@ -4466,7 +4466,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="88" spans="1:4">
+    <row r="88" spans="1:11">
       <c r="A88" s="1" t="s">
         <v>12</v>
       </c>
@@ -4474,7 +4474,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="89" spans="1:4">
+    <row r="89" spans="1:11">
       <c r="A89" s="1" t="s">
         <v>13</v>
       </c>
@@ -4482,31 +4482,55 @@
         <v>51</v>
       </c>
     </row>
-    <row r="90" spans="1:4">
+    <row r="90" spans="1:11">
       <c r="A90" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B90">
         <v>600</v>
       </c>
-    </row>
-    <row r="91" spans="1:4">
+      <c r="D90" s="11"/>
+      <c r="E90" s="11"/>
+      <c r="F90" s="11"/>
+      <c r="G90" s="11"/>
+      <c r="H90" s="11"/>
+      <c r="I90" s="11"/>
+      <c r="J90" s="11"/>
+      <c r="K90" s="11"/>
+    </row>
+    <row r="91" spans="1:11">
       <c r="A91" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B91">
         <v>35</v>
       </c>
-    </row>
-    <row r="92" spans="1:4">
+      <c r="D91" s="11"/>
+      <c r="E91" s="11"/>
+      <c r="F91" s="11"/>
+      <c r="G91" s="11"/>
+      <c r="H91" s="11"/>
+      <c r="I91" s="11"/>
+      <c r="J91" s="11"/>
+      <c r="K91" s="11"/>
+    </row>
+    <row r="92" spans="1:11">
       <c r="A92" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B92">
         <v>330</v>
       </c>
-    </row>
-    <row r="93" spans="1:4">
+      <c r="D92" s="11"/>
+      <c r="E92" s="11"/>
+      <c r="F92" s="11"/>
+      <c r="G92" s="11"/>
+      <c r="H92" s="11"/>
+      <c r="I92" s="11"/>
+      <c r="J92" s="11"/>
+      <c r="K92" s="11"/>
+    </row>
+    <row r="93" spans="1:11">
       <c r="A93" s="1" t="s">
         <v>2</v>
       </c>
@@ -4514,7 +4538,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="94" spans="1:4">
+    <row r="94" spans="1:11">
       <c r="A94" s="1" t="s">
         <v>3</v>
       </c>
@@ -4522,7 +4546,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="95" spans="1:4">
+    <row r="95" spans="1:11">
       <c r="A95" s="1" t="s">
         <v>4</v>
       </c>
@@ -4530,7 +4554,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="96" spans="1:4">
+    <row r="96" spans="1:11">
       <c r="A96" s="1" t="s">
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
added additional reason for lower % speedup in gRPC, hypothesis, which requires testing still
</commit_message>
<xml_diff>
--- a/results/concurrency/ConcurrencyActualResults.xlsx
+++ b/results/concurrency/ConcurrencyActualResults.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\audricho\Documents\ForOfficialDemo\results\concurrency\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78B1E355-37DF-4DC7-959C-AEAC66D832D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF2859E8-DC00-4401-AA03-240C7C1EB71B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="832" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="833" uniqueCount="47">
   <si>
     <t>stubGRPCPeoplePeopleInfoServiceStub P-R</t>
   </si>
@@ -205,6 +205,9 @@
   <si>
     <t>speedup not as sig also likely due to db not parallised so call and receive big data from db bottlenecked since large data already take up a lot of time so 20 calls at once will just end up being queued and bottlenecked there, not as much gap free time already prevopusly due to large payload size</t>
   </si>
+  <si>
+    <t>speedup not as high % for gRPC due to it reaching the limit of speed already, closer to speed limit bottlenecks due to stuff like db and backend threads etc, so less "space" to improve upon as well, while REST got more "space" to improve, since its further away from the speed limit bottleneck, =&gt; ie. speed limit constant is "x", the time taken now is (protocol+payload type parse/conversion time) + x, so tending closer to x so % increase is lesser and lesser, especially % wise since x/(0.1+x) can be very close to 1 is 0.1 &lt;&lt; x, so maybe need to time the "x" time taken but this is only so for single threaded backend, if backend multiple threads a bit hard unless time*thread/calls or something but if backend is single thread, sequential then backend just get "delay" due to db and backend by timing it, the entire process, then minus it away, but need to be careful not to count parsing or conversion into delay or something? ensure only db or backend single thread processes delay is counted towards it or something?</t>
+  </si>
 </sst>
 </file>
 
@@ -283,7 +286,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -303,15 +306,8 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -319,6 +315,12 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3633,7 +3635,6 @@
       <c r="B59">
         <v>52</v>
       </c>
-      <c r="P59" s="11"/>
     </row>
     <row r="60" spans="1:19">
       <c r="A60" s="1" t="s">
@@ -3782,10 +3783,10 @@
         <f>AVERAGE(I61:S61)</f>
         <v>0.67994783620603405</v>
       </c>
-      <c r="J62" s="7" t="s">
+      <c r="J62" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="K62" s="7"/>
+      <c r="K62" s="16"/>
       <c r="L62" s="2"/>
       <c r="M62" s="2"/>
       <c r="N62" s="2"/>
@@ -3802,13 +3803,13 @@
       <c r="B63">
         <v>330</v>
       </c>
-      <c r="D63" s="8" t="s">
+      <c r="D63" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="E63" s="8"/>
-      <c r="F63" s="8"/>
-      <c r="G63" s="8"/>
-      <c r="H63" s="8"/>
+      <c r="E63" s="17"/>
+      <c r="F63" s="17"/>
+      <c r="G63" s="17"/>
+      <c r="H63" s="17"/>
       <c r="I63" s="2">
         <f>(I60-$E$60)/$E$60</f>
         <v>0.57469015003261581</v>
@@ -3861,13 +3862,13 @@
       <c r="B64">
         <v>260</v>
       </c>
-      <c r="D64" s="8" t="s">
+      <c r="D64" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="E64" s="8"/>
-      <c r="F64" s="8"/>
-      <c r="G64" s="8"/>
-      <c r="H64" s="8"/>
+      <c r="E64" s="17"/>
+      <c r="F64" s="17"/>
+      <c r="G64" s="17"/>
+      <c r="H64" s="17"/>
       <c r="I64" s="2">
         <f>(I60-$E$60)/I60</f>
         <v>0.36495443247721626</v>
@@ -3936,7 +3937,7 @@
       <c r="B67">
         <v>629</v>
       </c>
-      <c r="D67" s="14" t="s">
+      <c r="D67" s="11" t="s">
         <v>36</v>
       </c>
     </row>
@@ -4014,49 +4015,49 @@
       <c r="D70" t="s">
         <v>28</v>
       </c>
-      <c r="E70" s="12">
+      <c r="E70" s="9">
         <v>30.66</v>
       </c>
-      <c r="F70" s="13">
+      <c r="F70" s="10">
         <v>309.27999999999997</v>
       </c>
-      <c r="G70" s="10">
+      <c r="G70" s="8">
         <v>329.9</v>
       </c>
-      <c r="H70" s="9">
+      <c r="H70" s="7">
         <v>260.88</v>
       </c>
-      <c r="I70" s="12">
+      <c r="I70" s="9">
         <v>48.28</v>
       </c>
-      <c r="J70" s="12">
+      <c r="J70" s="9">
         <v>50.86</v>
       </c>
-      <c r="K70" s="13">
+      <c r="K70" s="10">
         <v>601.62</v>
       </c>
-      <c r="L70" s="13">
+      <c r="L70" s="10">
         <v>597.16</v>
       </c>
-      <c r="M70" s="9">
+      <c r="M70" s="7">
         <v>285.2</v>
       </c>
-      <c r="N70" s="9">
+      <c r="N70" s="7">
         <v>279.3</v>
       </c>
-      <c r="O70" s="10">
+      <c r="O70" s="8">
         <v>410.24</v>
       </c>
-      <c r="P70" s="10">
+      <c r="P70" s="8">
         <v>402.88</v>
       </c>
-      <c r="Q70" s="12">
+      <c r="Q70" s="9">
         <v>50.02</v>
       </c>
-      <c r="R70" s="12">
+      <c r="R70" s="9">
         <v>50.5</v>
       </c>
-      <c r="S70" s="13">
+      <c r="S70" s="10">
         <v>597.44000000000005</v>
       </c>
     </row>
@@ -4113,7 +4114,7 @@
         <v>0.79687292964091694</v>
       </c>
       <c r="F75">
-        <f t="shared" ref="F74:S75" si="1">(F$69-F$70)/F$69</f>
+        <f t="shared" ref="F75:S75" si="1">(F$69-F$70)/F$69</f>
         <v>0.75401256661099181</v>
       </c>
       <c r="G75">
@@ -4184,7 +4185,7 @@
         <v>3.9230267449445533</v>
       </c>
       <c r="F76">
-        <f t="shared" ref="F75:S76" si="2">(F$69-F$70)/F$70</f>
+        <f t="shared" ref="F76:S76" si="2">(F$69-F$70)/F$70</f>
         <v>3.0652483186756339</v>
       </c>
       <c r="G76">
@@ -4269,63 +4270,63 @@
       <c r="D79" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E79" s="12">
+      <c r="E79" s="9">
         <f>E$70/E$69</f>
         <v>0.20312707035908309</v>
       </c>
-      <c r="F79" s="15">
+      <c r="F79" s="12">
         <f t="shared" ref="F79:S79" si="3">F$70/F$69</f>
         <v>0.24598743338900819</v>
       </c>
-      <c r="G79" s="10">
+      <c r="G79" s="8">
         <f t="shared" si="3"/>
         <v>0.28443578424610289</v>
       </c>
-      <c r="H79" s="9">
+      <c r="H79" s="7">
         <f t="shared" si="3"/>
         <v>0.55622361519764618</v>
       </c>
-      <c r="I79" s="12">
+      <c r="I79" s="9">
         <f t="shared" si="3"/>
         <v>0.1916481422673865</v>
       </c>
-      <c r="J79" s="12">
+      <c r="J79" s="9">
         <f t="shared" si="3"/>
         <v>0.20810147299509002</v>
       </c>
-      <c r="K79" s="13">
+      <c r="K79" s="10">
         <f t="shared" si="3"/>
         <v>0.26817330837122222</v>
       </c>
-      <c r="L79" s="13">
+      <c r="L79" s="10">
         <f t="shared" si="3"/>
         <v>0.26559094831036906</v>
       </c>
-      <c r="M79" s="9">
+      <c r="M79" s="7">
         <f t="shared" si="3"/>
         <v>0.32692924939245266</v>
       </c>
-      <c r="N79" s="16">
+      <c r="N79" s="13">
         <f t="shared" si="3"/>
         <v>0.32130777903043972</v>
       </c>
-      <c r="O79" s="10">
+      <c r="O79" s="8">
         <f t="shared" si="3"/>
         <v>0.26042354375095222</v>
       </c>
-      <c r="P79" s="17">
+      <c r="P79" s="14">
         <f t="shared" si="3"/>
         <v>0.2568012034369343</v>
       </c>
-      <c r="Q79" s="18">
+      <c r="Q79" s="15">
         <f t="shared" si="3"/>
         <v>0.1700319532259161</v>
       </c>
-      <c r="R79" s="12">
+      <c r="R79" s="9">
         <f t="shared" si="3"/>
         <v>0.18997818072379807</v>
       </c>
-      <c r="S79" s="13">
+      <c r="S79" s="10">
         <f t="shared" si="3"/>
         <v>0.29054126343432379</v>
       </c>
@@ -4340,68 +4341,68 @@
       <c r="D80" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E80" s="12">
+      <c r="E80" s="9">
         <f>E$69/E$70</f>
         <v>4.9230267449445533</v>
       </c>
-      <c r="F80" s="15">
+      <c r="F80" s="12">
         <f t="shared" ref="F80:S80" si="4">F$69/F$70</f>
         <v>4.0652483186756339</v>
       </c>
-      <c r="G80" s="10">
+      <c r="G80" s="8">
         <f t="shared" si="4"/>
         <v>3.515732040012125</v>
       </c>
-      <c r="H80" s="9">
+      <c r="H80" s="7">
         <f t="shared" si="4"/>
         <v>1.7978380864765409</v>
       </c>
-      <c r="I80" s="12">
+      <c r="I80" s="9">
         <f t="shared" si="4"/>
         <v>5.2178956089478037</v>
       </c>
-      <c r="J80" s="12">
+      <c r="J80" s="9">
         <f t="shared" si="4"/>
         <v>4.8053480141565084</v>
       </c>
-      <c r="K80" s="13">
+      <c r="K80" s="10">
         <f t="shared" si="4"/>
         <v>3.7289318839134338</v>
       </c>
-      <c r="L80" s="13">
+      <c r="L80" s="10">
         <f t="shared" si="4"/>
         <v>3.7651885591801197</v>
       </c>
-      <c r="M80" s="9">
+      <c r="M80" s="7">
         <f t="shared" si="4"/>
         <v>3.0587657784011224</v>
       </c>
-      <c r="N80" s="16">
+      <c r="N80" s="13">
         <f t="shared" si="4"/>
         <v>3.1122807017543859</v>
       </c>
-      <c r="O80" s="10">
+      <c r="O80" s="8">
         <f t="shared" si="4"/>
         <v>3.8398985959438376</v>
       </c>
-      <c r="P80" s="17">
+      <c r="P80" s="14">
         <f t="shared" si="4"/>
         <v>3.8940627482128671</v>
       </c>
-      <c r="Q80" s="18">
+      <c r="Q80" s="15">
         <f t="shared" si="4"/>
         <v>5.8812475009996001</v>
       </c>
-      <c r="R80" s="12">
+      <c r="R80" s="9">
         <f t="shared" si="4"/>
         <v>5.263762376237624</v>
       </c>
-      <c r="S80" s="13">
+      <c r="S80" s="10">
         <f t="shared" si="4"/>
         <v>3.4418519014461704</v>
       </c>
     </row>
-    <row r="81" spans="1:11">
+    <row r="81" spans="1:4">
       <c r="A81" s="1" t="s">
         <v>5</v>
       </c>
@@ -4409,7 +4410,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="82" spans="1:11">
+    <row r="82" spans="1:4">
       <c r="A82" s="1" t="s">
         <v>6</v>
       </c>
@@ -4417,7 +4418,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="83" spans="1:11">
+    <row r="83" spans="1:4">
       <c r="A83" s="1" t="s">
         <v>7</v>
       </c>
@@ -4425,7 +4426,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="84" spans="1:11">
+    <row r="84" spans="1:4">
       <c r="A84" s="1" t="s">
         <v>8</v>
       </c>
@@ -4436,7 +4437,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="85" spans="1:11">
+    <row r="85" spans="1:4">
       <c r="A85" s="1" t="s">
         <v>9</v>
       </c>
@@ -4447,7 +4448,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="86" spans="1:11">
+    <row r="86" spans="1:4">
       <c r="A86" s="1" t="s">
         <v>10</v>
       </c>
@@ -4458,15 +4459,18 @@
         <v>45</v>
       </c>
     </row>
-    <row r="87" spans="1:11">
+    <row r="87" spans="1:4">
       <c r="A87" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B87">
         <v>382</v>
       </c>
-    </row>
-    <row r="88" spans="1:11">
+      <c r="D87" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4">
       <c r="A88" s="1" t="s">
         <v>12</v>
       </c>
@@ -4474,7 +4478,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="89" spans="1:11">
+    <row r="89" spans="1:4">
       <c r="A89" s="1" t="s">
         <v>13</v>
       </c>
@@ -4482,55 +4486,31 @@
         <v>51</v>
       </c>
     </row>
-    <row r="90" spans="1:11">
+    <row r="90" spans="1:4">
       <c r="A90" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B90">
         <v>600</v>
       </c>
-      <c r="D90" s="11"/>
-      <c r="E90" s="11"/>
-      <c r="F90" s="11"/>
-      <c r="G90" s="11"/>
-      <c r="H90" s="11"/>
-      <c r="I90" s="11"/>
-      <c r="J90" s="11"/>
-      <c r="K90" s="11"/>
-    </row>
-    <row r="91" spans="1:11">
+    </row>
+    <row r="91" spans="1:4">
       <c r="A91" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B91">
         <v>35</v>
       </c>
-      <c r="D91" s="11"/>
-      <c r="E91" s="11"/>
-      <c r="F91" s="11"/>
-      <c r="G91" s="11"/>
-      <c r="H91" s="11"/>
-      <c r="I91" s="11"/>
-      <c r="J91" s="11"/>
-      <c r="K91" s="11"/>
-    </row>
-    <row r="92" spans="1:11">
+    </row>
+    <row r="92" spans="1:4">
       <c r="A92" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B92">
         <v>330</v>
       </c>
-      <c r="D92" s="11"/>
-      <c r="E92" s="11"/>
-      <c r="F92" s="11"/>
-      <c r="G92" s="11"/>
-      <c r="H92" s="11"/>
-      <c r="I92" s="11"/>
-      <c r="J92" s="11"/>
-      <c r="K92" s="11"/>
-    </row>
-    <row r="93" spans="1:11">
+    </row>
+    <row r="93" spans="1:4">
       <c r="A93" s="1" t="s">
         <v>2</v>
       </c>
@@ -4538,7 +4518,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="94" spans="1:11">
+    <row r="94" spans="1:4">
       <c r="A94" s="1" t="s">
         <v>3</v>
       </c>
@@ -4546,7 +4526,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="95" spans="1:11">
+    <row r="95" spans="1:4">
       <c r="A95" s="1" t="s">
         <v>4</v>
       </c>
@@ -4554,7 +4534,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="96" spans="1:11">
+    <row r="96" spans="1:4">
       <c r="A96" s="1" t="s">
         <v>5</v>
       </c>

</xml_diff>